<commit_message>
fix: add a Code column to the Tunisia vendor bill layout
The Tunisian frame sizes column A for Code and B for Désignation (the
VAT recap beneath shares them), but the incoming invoice was the only
type without a Code column, so descriptions wrapped into the narrow
column A and overflowed onto the rows below. Join the linked
product's SKU onto incoming invoice line items (the same LEFT JOIN
purchase orders use), expose it as {{lineItems.sku}}, and lead the
Tunisia bill table with Code like every other type.
</commit_message>
<xml_diff>
--- a/db/templates/incoming_invoice_default.xlsx
+++ b/db/templates/incoming_invoice_default.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
   <si>
     <t>{{vendor.name}}</t>
   </si>
@@ -291,6 +291,12 @@
   </si>
   <si>
     <t>Marker (not a value) — place alone in one cell of the row to repeat once per line item</t>
+  </si>
+  <si>
+    <t>{{lineItems.sku}}</t>
+  </si>
+  <si>
+    <t>Linked product's SKU (the Code column), blank on a free-text line</t>
   </si>
   <si>
     <t>Line item description</t>
@@ -1187,54 +1193,54 @@
     </row>
     <row r="34">
       <c r="B34" t="s">
-        <v>21</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="s">
         <v>25</v>
       </c>
-      <c r="C38" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="s">
-        <v>95</v>
+      <c r="C39" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="40">
-      <c r="B40" t="s">
-        <v>96</v>
-      </c>
-      <c r="C40" t="s">
+      <c r="A40" s="12" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1263,52 +1269,52 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="s">
+      <c r="B44" t="s">
         <v>104</v>
       </c>
+      <c r="C44" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="45">
-      <c r="B45" t="s">
-        <v>28</v>
-      </c>
-      <c r="C45" t="s">
-        <v>105</v>
+      <c r="A45" s="12" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C46" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C47" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" t="s">
-        <v>108</v>
+        <v>32</v>
       </c>
       <c r="C48" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="s">
+      <c r="B49" t="s">
         <v>110</v>
       </c>
+      <c r="C49" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="50">
-      <c r="B50" t="s">
-        <v>111</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="A50" s="12" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1326,6 +1332,14 @@
       </c>
       <c r="C52" t="s">
         <v>116</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="s">
+        <v>117</v>
+      </c>
+      <c r="C53" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1333,9 +1347,9 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A50:C50"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>